<commit_message>
Projeto Flask Mostruário Digital CLAMI
</commit_message>
<xml_diff>
--- a/data/CATALAGO MOSTRUARIO DIGITAL.xlsx
+++ b/data/CATALAGO MOSTRUARIO DIGITAL.xlsx
@@ -5,19 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\22_MOSTRUARIO DIGITAL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\22_MOSTRUARIO DIGITAL\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C64ACB94-58ED-4CD2-8745-4B5F631A144C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{352D2227-969D-4118-9365-9531AD1B5A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="produtos" sheetId="1" r:id="rId1"/>
     <sheet name="95" sheetId="3" r:id="rId2"/>
     <sheet name="138" sheetId="4" r:id="rId3"/>
     <sheet name="3992" sheetId="2" r:id="rId4"/>
-    <sheet name="12401" sheetId="5" r:id="rId5"/>
+    <sheet name="10202" sheetId="6" r:id="rId5"/>
+    <sheet name="12401" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="501">
   <si>
     <t xml:space="preserve">ALUMINIO </t>
   </si>
@@ -805,6 +806,744 @@
   </si>
   <si>
     <t>CADEIRA GENEBRA</t>
+  </si>
+  <si>
+    <t>APARADOR THAE</t>
+  </si>
+  <si>
+    <t>APARADOR VELL 01</t>
+  </si>
+  <si>
+    <t>BANQUETA BAR</t>
+  </si>
+  <si>
+    <t>BANQUETA BAR THAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUFFET </t>
+  </si>
+  <si>
+    <t>BUFFET HOLLIE MACICO</t>
+  </si>
+  <si>
+    <t>BUFFET THAE</t>
+  </si>
+  <si>
+    <t>CADEIRA KEEF</t>
+  </si>
+  <si>
+    <t>ESCRIVANINHA</t>
+  </si>
+  <si>
+    <t>ESCRIVANINHA DESKA</t>
+  </si>
+  <si>
+    <t>HOME</t>
+  </si>
+  <si>
+    <t>MESA JANTAR THAE</t>
+  </si>
+  <si>
+    <t>MESA JANTAR VELL</t>
+  </si>
+  <si>
+    <t>MOVEL BAR</t>
+  </si>
+  <si>
+    <t>MOVEL BAR HOLLIE MACICO</t>
+  </si>
+  <si>
+    <t>HOME THAE</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_APARADOR THAE.jpg</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_APARADOR_VELL.jpg</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_BANQUETA BAR THAE.jpg</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_BUFFET THAE.png</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_BUFFET HOLLIE.jpg</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_CADEIRA KEEF C-BRACO.jpg</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_ESCRIVANINHA DESKA.jpg</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_HOME THAE.jpg</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_MESA_JANTAR_VELL.jpg</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_MESA JANTAR THAE.jpg</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\PRODUTOS\10202\10202_MOVEL BAR HOLLIE.jpg</t>
+  </si>
+  <si>
+    <t>RECOURO</t>
+  </si>
+  <si>
+    <t>LAMINA IMBUIA</t>
+  </si>
+  <si>
+    <t>RECOURO CAMEL</t>
+  </si>
+  <si>
+    <t>RECOURO PRETO</t>
+  </si>
+  <si>
+    <t>RECOURO PINHAO</t>
+  </si>
+  <si>
+    <t>COURO CLASSE 2</t>
+  </si>
+  <si>
+    <t>COURO CARAMELO (CL2)</t>
+  </si>
+  <si>
+    <t>COURO PEROLA (CL2)</t>
+  </si>
+  <si>
+    <t>COURO AVELA (CL2)</t>
+  </si>
+  <si>
+    <t>COURO CLASSE 3</t>
+  </si>
+  <si>
+    <t>COURO PRETO (CL3)</t>
+  </si>
+  <si>
+    <t>COURO MUSGO (CL3)</t>
+  </si>
+  <si>
+    <t>COURO NUDE (CL3)</t>
+  </si>
+  <si>
+    <t>COURO NAVY (CL3)</t>
+  </si>
+  <si>
+    <t>COURO CINZA (CL3)</t>
+  </si>
+  <si>
+    <t>COURO CLASSE 4</t>
+  </si>
+  <si>
+    <t>COURO GRIS (CL4)</t>
+  </si>
+  <si>
+    <t>COURO PINHAO (CL4)</t>
+  </si>
+  <si>
+    <t>COURO COFFEE (CL4)</t>
+  </si>
+  <si>
+    <t>COURO NERO (CL4)</t>
+  </si>
+  <si>
+    <t>COURO CAMEL (CL4)</t>
+  </si>
+  <si>
+    <t>COURO CLASSE 5</t>
+  </si>
+  <si>
+    <t>CAMURCA BRULLE (CL5)</t>
+  </si>
+  <si>
+    <t>CAMURCA MARROQUINO (CL5)</t>
+  </si>
+  <si>
+    <t>CAMURCA ARGILA (CL5)</t>
+  </si>
+  <si>
+    <t>CAMURCA VERDE (CL5)</t>
+  </si>
+  <si>
+    <t>MARMORE</t>
+  </si>
+  <si>
+    <t>MARMORE BRANCO CARRARA</t>
+  </si>
+  <si>
+    <t>MARMORE NERO MARQUINA</t>
+  </si>
+  <si>
+    <t>MARMORE ROSA PARANA</t>
+  </si>
+  <si>
+    <t>ACO CARBONO</t>
+  </si>
+  <si>
+    <t>ACO CARBONO MTZ CHAMPAGNE</t>
+  </si>
+  <si>
+    <t>ACO CARBONO GOLD</t>
+  </si>
+  <si>
+    <t>ACO CARBONO COOPER</t>
+  </si>
+  <si>
+    <t>ACO CARBONO URANO</t>
+  </si>
+  <si>
+    <t>ACO CARBONO MARROM PEROLIZADO</t>
+  </si>
+  <si>
+    <t>ACO CARBONO PRETO TEXTURIZADO</t>
+  </si>
+  <si>
+    <t>ACO CARBONO GRAY</t>
+  </si>
+  <si>
+    <t>ACO CARBONO MARROM FOSCO</t>
+  </si>
+  <si>
+    <t>ACO CARBONO FLOOR</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ NATURAL</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING NOGUEIRA</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING FREIJO</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING CLOUD</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING NUDE</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING FENDI</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING SMOKE</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING GREEN</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING INDIGO</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING DARK WALNUT</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING EBANIZADO</t>
+  </si>
+  <si>
+    <t>MADEIRA JEQ TING MTZ SILVER</t>
+  </si>
+  <si>
+    <t>LAMINA CARVALHO</t>
+  </si>
+  <si>
+    <t>LAMINA CARV NATURAL</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING NOGUEIRA</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING FREIJO</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING CLOUD</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING NUDE</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING FENDI</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING SMOKE</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING GREEN</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING INDIGO</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING DARK WALNUT</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING EBANIZADO</t>
+  </si>
+  <si>
+    <t>LAMINA CARV TING MTZ SILVER</t>
+  </si>
+  <si>
+    <t>LAMINA JEQUITIBA</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ NATURAL</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING NOGUEIRA</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING FREIJO</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING CLOUD</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING NUDE</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING FENDI</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING SMOKE</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING GREEN</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING INDIGO</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING DARK WALNUT</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING EBANIZADO</t>
+  </si>
+  <si>
+    <t>LAMINA JEQ TING MTZ SILVER</t>
+  </si>
+  <si>
+    <t>LAMINA NATURAL</t>
+  </si>
+  <si>
+    <t>LAMINA NOGUEIRA NATURAL</t>
+  </si>
+  <si>
+    <t>MADEIRA FAIA NATURAL</t>
+  </si>
+  <si>
+    <t>TELA SEXTAVADA ALG NATURAL</t>
+  </si>
+  <si>
+    <t>TELA SEXTAVADA ALG NOGUEIRA</t>
+  </si>
+  <si>
+    <t>TELA SEXTAVADA ALG JEQUITIBA</t>
+  </si>
+  <si>
+    <t>TELA SEXTAVADA ALG EBANIZADA</t>
+  </si>
+  <si>
+    <t>TELA SEXTAVADA RATTAN NATURAL</t>
+  </si>
+  <si>
+    <t>TELA QUADRICULADA</t>
+  </si>
+  <si>
+    <t>TELA QUAD RATTAN NATURAL RC07</t>
+  </si>
+  <si>
+    <t>LAMINA FAIA</t>
+  </si>
+  <si>
+    <t>LAMINA FAIA NATURAL</t>
+  </si>
+  <si>
+    <t>MADEIRA IMBUIA NATURAL</t>
+  </si>
+  <si>
+    <t>LAMINA IMBUIA NATURAL</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO NATURAL</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING NOGUEIRA</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING FREIJO</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING CLOUD</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING NUDE</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING FENDI</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING SMOKE</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING GREEN</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING INDIGO</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING DARK WALNUT</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING EBANIZADO</t>
+  </si>
+  <si>
+    <t>MADEIRA ECO TING SILVER</t>
+  </si>
+  <si>
+    <t>DEKTON</t>
+  </si>
+  <si>
+    <t>APENAS ENCOSTO</t>
+  </si>
+  <si>
+    <t>AURA</t>
+  </si>
+  <si>
+    <t>KELYA</t>
+  </si>
+  <si>
+    <t>MADEIRA TING JEQUITIBA</t>
+  </si>
+  <si>
+    <t>LAMINA FREIJO NATURAL</t>
+  </si>
+  <si>
+    <t>FREIJO NATURAL</t>
+  </si>
+  <si>
+    <t>MADEIRA FREIJO</t>
+  </si>
+  <si>
+    <t>MADEIRA FAIA</t>
+  </si>
+  <si>
+    <t>MADEIRA IMBUIA</t>
+  </si>
+  <si>
+    <t>MADEIRA  ECOGRANDIS</t>
+  </si>
+  <si>
+    <t>APARADOR THAE ECOGRANDIS</t>
+  </si>
+  <si>
+    <t>MESA JANTAR THAE ECOGRANDIS</t>
+  </si>
+  <si>
+    <t>ECO - LAMINA CARVALHO</t>
+  </si>
+  <si>
+    <t>ECO - LAMINA NATURAL</t>
+  </si>
+  <si>
+    <t>ACRESCIMO DE 10%</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA FAIA NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA IMBUIA NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING CLOUD.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING DARK WALNUT.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING EBANIZADO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING FENDI.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING FREIJO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING GREEN.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING INDIGO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING MTZ SILVER.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING NOGUEIRA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING NUDE.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA JEQ TING SMOKE.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING CLOUD.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING DARK WALNUT.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING EBANIZADO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING FENDI.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING FREIJO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING GREEN.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING INDIGO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING NOGUEIRA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING NUDE.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING SILVER.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MADEIRA ECO TING SMOKE.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA FAIA NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA IMBUIA NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA NOGUEIRA NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING CLOUD.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING DARK WALNUT.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING EBANIZADO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING FENDI.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING FREIJO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING GREEN.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING INDIGO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING MTZ SILVER.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING NOGUEIRA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING NUDE.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA JEQ TING SMOKE.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING CLOUD.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING DARK WALNUT.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING EBANIZADO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING FENDI.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING FREIJO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING GREEN.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING INDIGO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING MTZ SILVER.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING NOGUEIRA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING NUDE.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\LAMINA CARV TING SMOKE.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MARMORE BRANCO CARRARA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MARMORE NERO MARQUINA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\MARMORE ROSA PARANA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\ACO CARBONO COOPER.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\ACO CARBONO FLOOR.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\ACO CARBONO GOLD.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\ACO CARBONO GRAY.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\ACO CARBONO MARROM FOSCO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\ACO CARBONO MARROM PEROLIZADO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\ACO CARBONO MTZ CHAMPAGNE.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\ACO CARBONO PRETO TEXTURIZADO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\ACO CARBONO URANO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO AVELA (CL2).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO CAMEL (CL4).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO CARAMELO (CL2).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO CINZA (CL3).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO COFFEE (CL4).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO GRIS (CL4).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO MUSGO (CL3).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO NAVY (CL3).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO NERO (CL4).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO NUDE (CL3).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO PEROLA (CL2).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO PINHAO (CL4).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\COURO PRETO (CL3).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\CAMURCA ARGILA (CL5).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\CAMURCA BRULLE (CL5).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\CAMURCA MARROQUINO (CL5).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\CAMURCA VERDE (CL5).JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\RECOURO CAMEL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\RECOURO PINHAO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\RECOURO PRETO.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\TELA QUAD RATTAN NATURAL RC07.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\TELA SEXTAVADA ALG EBANIZADA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\TELA SEXTAVADA ALG JEQUITIBA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\TELA SEXTAVADA ALG NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\TELA SEXTAVADA ALG NOGUEIRA.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\TELA SEXTAVADA RATTAN NATURAL.JPG</t>
+  </si>
+  <si>
+    <t>TRANCADO</t>
+  </si>
+  <si>
+    <t>TRANCADO CHESS</t>
+  </si>
+  <si>
+    <t>TRANCADO KAED</t>
+  </si>
+  <si>
+    <t>TRANCADO PIETRO</t>
+  </si>
+  <si>
+    <t>ACRESCIMO DE 20%</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\TRANCADO CHESS.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\TRANCADO KAED.JPG</t>
+  </si>
+  <si>
+    <t>P:\22_MOSTRUARIO DIGITAL\static\ACABAMENTOS\10202\TRANCADO PIETRO.JPG</t>
   </si>
 </sst>
 </file>
@@ -865,7 +1604,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -902,6 +1641,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -930,7 +1675,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -999,6 +1744,44 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1306,15 +2089,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:F118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" customWidth="1"/>
     <col min="2" max="2" width="19.140625" customWidth="1"/>
     <col min="3" max="3" width="36.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="88.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.85546875" customWidth="1"/>
+    <col min="6" max="6" width="43.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1501,7 +2284,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <v>95</v>
       </c>
@@ -1518,19 +2301,19 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16"/>
       <c r="D18" s="10" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="D19" s="10" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <v>95</v>
       </c>
@@ -1547,16 +2330,16 @@
         <v>110</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="D21" s="10" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="13">
         <v>138</v>
       </c>
@@ -1573,22 +2356,22 @@
         <v>127</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13"/>
       <c r="D24" s="19" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="13"/>
       <c r="D25" s="19" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
     </row>
-    <row r="27" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="13">
         <v>3992</v>
       </c>
@@ -1605,81 +2388,887 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="16"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="23">
+    <row r="28" spans="1:6" s="41" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="40"/>
+    </row>
+    <row r="29" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B29" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="43" t="s">
+        <v>397</v>
+      </c>
+      <c r="D29" s="43" t="s">
+        <v>396</v>
+      </c>
+      <c r="E29" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="F29" s="12"/>
+    </row>
+    <row r="30" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="42"/>
+      <c r="B30" s="43"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E30" s="43"/>
+      <c r="F30" s="12"/>
+    </row>
+    <row r="31" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="42"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="43" t="s">
+        <v>399</v>
+      </c>
+      <c r="E31" s="43"/>
+      <c r="F31" s="12"/>
+    </row>
+    <row r="32" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="42"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43" t="s">
+        <v>400</v>
+      </c>
+      <c r="E32" s="43"/>
+      <c r="F32" s="12"/>
+    </row>
+    <row r="33" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="42"/>
+      <c r="B33" s="43"/>
+      <c r="C33" s="43"/>
+      <c r="D33" s="43" t="s">
+        <v>308</v>
+      </c>
+      <c r="E33" s="43"/>
+      <c r="F33" s="12"/>
+    </row>
+    <row r="34" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="42"/>
+      <c r="B34" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="43" t="s">
+        <v>255</v>
+      </c>
+      <c r="D34" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E34" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="F34" s="12"/>
+    </row>
+    <row r="35" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="42"/>
+      <c r="B35" s="43"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E35" s="43"/>
+      <c r="F35" s="12"/>
+    </row>
+    <row r="36" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="42"/>
+      <c r="B36" s="43"/>
+      <c r="C36" s="43"/>
+      <c r="D36" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E36" s="43"/>
+      <c r="F36" s="12"/>
+    </row>
+    <row r="37" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="42"/>
+      <c r="B37" s="43"/>
+      <c r="C37" s="43"/>
+      <c r="D37" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="E37" s="43"/>
+      <c r="F37" s="12"/>
+    </row>
+    <row r="38" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="42"/>
+      <c r="B38" s="43"/>
+      <c r="C38" s="43"/>
+      <c r="D38" s="43" t="s">
+        <v>308</v>
+      </c>
+      <c r="E38" s="43"/>
+      <c r="F38" s="12"/>
+    </row>
+    <row r="39" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="42"/>
+      <c r="B39" s="43"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43" t="s">
+        <v>395</v>
+      </c>
+      <c r="E39" s="43"/>
+      <c r="F39" s="12"/>
+    </row>
+    <row r="40" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="42"/>
+      <c r="B40" s="43"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43" t="s">
+        <v>283</v>
+      </c>
+      <c r="E40" s="43"/>
+      <c r="F40" s="12"/>
+    </row>
+    <row r="41" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B41" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="C41" s="43" t="s">
+        <v>256</v>
+      </c>
+      <c r="D41" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E41" s="43" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="42"/>
+      <c r="B42" s="43"/>
+      <c r="C42" s="43"/>
+      <c r="D42" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E42" s="43"/>
+    </row>
+    <row r="43" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="42"/>
+      <c r="B43" s="43"/>
+      <c r="C43" s="43"/>
+      <c r="D43" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E43" s="43"/>
+    </row>
+    <row r="44" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="42"/>
+      <c r="B44" s="43"/>
+      <c r="C44" s="43"/>
+      <c r="D44" s="43" t="s">
+        <v>312</v>
+      </c>
+      <c r="E44" s="43"/>
+    </row>
+    <row r="45" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="42"/>
+      <c r="B45" s="43"/>
+      <c r="C45" s="43"/>
+      <c r="D45" s="43" t="s">
+        <v>394</v>
+      </c>
+      <c r="E45" s="43"/>
+    </row>
+    <row r="46" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B46" s="43" t="s">
+        <v>257</v>
+      </c>
+      <c r="C46" s="43" t="s">
+        <v>258</v>
+      </c>
+      <c r="D46" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E46" s="43" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="42"/>
+      <c r="B47" s="43"/>
+      <c r="C47" s="43"/>
+      <c r="D47" s="43" t="s">
+        <v>312</v>
+      </c>
+      <c r="E47" s="43"/>
+    </row>
+    <row r="48" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="42"/>
+      <c r="B48" s="43"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43" t="s">
+        <v>233</v>
+      </c>
+      <c r="E48" s="43"/>
+    </row>
+    <row r="49" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="42"/>
+      <c r="B49" s="43"/>
+      <c r="C49" s="43"/>
+      <c r="D49" s="43" t="s">
+        <v>287</v>
+      </c>
+      <c r="E49" s="43"/>
+    </row>
+    <row r="50" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="42"/>
+      <c r="B50" s="43"/>
+      <c r="C50" s="43"/>
+      <c r="D50" s="43" t="s">
+        <v>291</v>
+      </c>
+      <c r="E50" s="43"/>
+    </row>
+    <row r="51" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="42"/>
+      <c r="B51" s="43"/>
+      <c r="C51" s="43"/>
+      <c r="D51" s="43" t="s">
+        <v>297</v>
+      </c>
+      <c r="E51" s="43"/>
+    </row>
+    <row r="52" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="42"/>
+      <c r="B52" s="43"/>
+      <c r="C52" s="43"/>
+      <c r="D52" s="43" t="s">
+        <v>303</v>
+      </c>
+      <c r="E52" s="43"/>
+    </row>
+    <row r="53" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B53" s="43" t="s">
+        <v>259</v>
+      </c>
+      <c r="C53" s="43" t="s">
+        <v>260</v>
+      </c>
+      <c r="D53" s="43" t="s">
+        <v>312</v>
+      </c>
+      <c r="E53" s="43" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="42"/>
+      <c r="B54" s="43"/>
+      <c r="C54" s="43"/>
+      <c r="D54" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E54" s="43"/>
+    </row>
+    <row r="55" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="42"/>
+      <c r="B55" s="43"/>
+      <c r="C55" s="43"/>
+      <c r="D55" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E55" s="43"/>
+    </row>
+    <row r="56" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="42"/>
+      <c r="B56" s="43"/>
+      <c r="C56" s="43"/>
+      <c r="D56" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E56" s="43"/>
+    </row>
+    <row r="57" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="42"/>
+      <c r="B57" s="43"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="E57" s="43"/>
+    </row>
+    <row r="58" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="42"/>
+      <c r="B58" s="43"/>
+      <c r="C58" s="43"/>
+      <c r="D58" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E58" s="43"/>
+    </row>
+    <row r="59" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="42"/>
+      <c r="B59" s="43"/>
+      <c r="C59" s="43"/>
+      <c r="D59" s="43" t="s">
+        <v>308</v>
+      </c>
+      <c r="E59" s="43"/>
+    </row>
+    <row r="60" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B60" s="43" t="s">
+        <v>259</v>
+      </c>
+      <c r="C60" s="43" t="s">
+        <v>261</v>
+      </c>
+      <c r="D60" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E60" s="43" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="42"/>
+      <c r="B61" s="43"/>
+      <c r="C61" s="43"/>
+      <c r="D61" s="43" t="s">
+        <v>395</v>
+      </c>
+      <c r="E61" s="43"/>
+    </row>
+    <row r="62" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="42"/>
+      <c r="B62" s="43"/>
+      <c r="C62" s="43"/>
+      <c r="D62" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E62" s="43"/>
+    </row>
+    <row r="63" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="42"/>
+      <c r="B63" s="43"/>
+      <c r="C63" s="43"/>
+      <c r="D63" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E63" s="43"/>
+    </row>
+    <row r="64" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="42"/>
+      <c r="B64" s="43"/>
+      <c r="C64" s="43"/>
+      <c r="D64" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="E64" s="43"/>
+    </row>
+    <row r="65" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="42"/>
+      <c r="B65" s="43"/>
+      <c r="C65" s="43"/>
+      <c r="D65" s="43" t="s">
+        <v>283</v>
+      </c>
+      <c r="E65" s="43"/>
+    </row>
+    <row r="66" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B66" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="C66" s="43" t="s">
+        <v>262</v>
+      </c>
+      <c r="D66" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E66" s="43" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="42"/>
+      <c r="B67" s="43"/>
+      <c r="C67" s="43"/>
+      <c r="D67" s="43" t="s">
+        <v>287</v>
+      </c>
+      <c r="E67" s="43"/>
+    </row>
+    <row r="68" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="42"/>
+      <c r="B68" s="43"/>
+      <c r="C68" s="43"/>
+      <c r="D68" s="43" t="s">
+        <v>291</v>
+      </c>
+      <c r="E68" s="43"/>
+    </row>
+    <row r="69" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="42"/>
+      <c r="B69" s="43"/>
+      <c r="C69" s="43"/>
+      <c r="D69" s="43" t="s">
+        <v>297</v>
+      </c>
+      <c r="E69" s="43"/>
+    </row>
+    <row r="70" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="42"/>
+      <c r="B70" s="43"/>
+      <c r="C70" s="43"/>
+      <c r="D70" s="43" t="s">
+        <v>303</v>
+      </c>
+      <c r="E70" s="43"/>
+    </row>
+    <row r="71" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B71" s="43" t="s">
+        <v>263</v>
+      </c>
+      <c r="C71" s="43" t="s">
+        <v>264</v>
+      </c>
+      <c r="D71" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E71" s="43" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="42"/>
+      <c r="B72" s="43"/>
+      <c r="C72" s="43"/>
+      <c r="D72" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E72" s="43"/>
+    </row>
+    <row r="73" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="42"/>
+      <c r="B73" s="43"/>
+      <c r="C73" s="43"/>
+      <c r="D73" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E73" s="43"/>
+    </row>
+    <row r="74" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="42"/>
+      <c r="B74" s="43"/>
+      <c r="C74" s="43"/>
+      <c r="D74" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="E74" s="43"/>
+    </row>
+    <row r="75" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="42"/>
+      <c r="B75" s="43"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43" t="s">
+        <v>283</v>
+      </c>
+      <c r="E75" s="43"/>
+    </row>
+    <row r="76" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="42"/>
+      <c r="B76" s="43"/>
+      <c r="C76" s="43"/>
+      <c r="D76" s="43" t="s">
+        <v>312</v>
+      </c>
+      <c r="E76" s="43"/>
+    </row>
+    <row r="77" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B77" s="43" t="s">
+        <v>265</v>
+      </c>
+      <c r="C77" s="43" t="s">
+        <v>270</v>
+      </c>
+      <c r="D77" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E77" s="43" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="42"/>
+      <c r="B78" s="43"/>
+      <c r="C78" s="43"/>
+      <c r="D78" s="43" t="s">
+        <v>395</v>
+      </c>
+      <c r="E78" s="43"/>
+    </row>
+    <row r="79" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="42"/>
+      <c r="B79" s="43"/>
+      <c r="C79" s="43"/>
+      <c r="D79" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E79" s="43"/>
+    </row>
+    <row r="80" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="42"/>
+      <c r="B80" s="43"/>
+      <c r="C80" s="43"/>
+      <c r="D80" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E80" s="43"/>
+    </row>
+    <row r="81" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="42"/>
+      <c r="B81" s="43"/>
+      <c r="C81" s="43"/>
+      <c r="D81" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="E81" s="43"/>
+    </row>
+    <row r="82" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="42"/>
+      <c r="B82" s="43"/>
+      <c r="C82" s="43"/>
+      <c r="D82" s="43" t="s">
+        <v>283</v>
+      </c>
+      <c r="E82" s="43"/>
+    </row>
+    <row r="83" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B83" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C83" s="43" t="s">
+        <v>398</v>
+      </c>
+      <c r="D83" s="43" t="s">
+        <v>396</v>
+      </c>
+      <c r="E83" s="43" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="42"/>
+      <c r="B84" s="43"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E84" s="43"/>
+    </row>
+    <row r="85" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="42"/>
+      <c r="B85" s="43"/>
+      <c r="C85" s="43"/>
+      <c r="D85" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E85" s="43"/>
+    </row>
+    <row r="86" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="42"/>
+      <c r="B86" s="43"/>
+      <c r="C86" s="43"/>
+      <c r="D86" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="E86" s="43"/>
+    </row>
+    <row r="87" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="42"/>
+      <c r="B87" s="43"/>
+      <c r="C87" s="43"/>
+      <c r="D87" s="43" t="s">
+        <v>308</v>
+      </c>
+      <c r="E87" s="43"/>
+    </row>
+    <row r="88" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="42"/>
+      <c r="B88" s="43"/>
+      <c r="C88" s="43" t="s">
+        <v>266</v>
+      </c>
+      <c r="D88" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E88" s="43" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="42"/>
+      <c r="B89" s="43"/>
+      <c r="C89" s="43"/>
+      <c r="D89" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E89" s="43"/>
+    </row>
+    <row r="90" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="42"/>
+      <c r="B90" s="43"/>
+      <c r="C90" s="43"/>
+      <c r="D90" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E90" s="43"/>
+    </row>
+    <row r="91" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="42"/>
+      <c r="B91" s="43"/>
+      <c r="C91" s="43"/>
+      <c r="D91" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="E91" s="43"/>
+    </row>
+    <row r="92" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="42"/>
+      <c r="B92" s="43"/>
+      <c r="C92" s="43"/>
+      <c r="D92" s="43" t="s">
+        <v>308</v>
+      </c>
+      <c r="E92" s="43"/>
+    </row>
+    <row r="93" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="42"/>
+      <c r="B93" s="43"/>
+      <c r="C93" s="43"/>
+      <c r="D93" s="43" t="s">
+        <v>395</v>
+      </c>
+      <c r="E93" s="43"/>
+    </row>
+    <row r="94" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="42"/>
+      <c r="B94" s="43"/>
+      <c r="C94" s="43"/>
+      <c r="D94" s="43" t="s">
+        <v>283</v>
+      </c>
+      <c r="E94" s="43"/>
+    </row>
+    <row r="95" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B95" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C95" s="43" t="s">
+        <v>267</v>
+      </c>
+      <c r="D95" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E95" s="43" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="42"/>
+      <c r="B96" s="43"/>
+      <c r="C96" s="43"/>
+      <c r="D96" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E96" s="43"/>
+    </row>
+    <row r="97" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="42"/>
+      <c r="B97" s="43"/>
+      <c r="C97" s="43"/>
+      <c r="D97" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E97" s="43"/>
+    </row>
+    <row r="98" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="42"/>
+      <c r="B98" s="43"/>
+      <c r="C98" s="43"/>
+      <c r="D98" s="43" t="s">
+        <v>312</v>
+      </c>
+      <c r="E98" s="43"/>
+    </row>
+    <row r="99" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="42">
+        <v>10202</v>
+      </c>
+      <c r="B99" s="43" t="s">
+        <v>268</v>
+      </c>
+      <c r="C99" s="43" t="s">
+        <v>269</v>
+      </c>
+      <c r="D99" s="43" t="s">
+        <v>312</v>
+      </c>
+      <c r="E99" s="43" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="42"/>
+      <c r="B100" s="43"/>
+      <c r="C100" s="43"/>
+      <c r="D100" s="43" t="s">
+        <v>390</v>
+      </c>
+      <c r="E100" s="43"/>
+    </row>
+    <row r="101" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="42"/>
+      <c r="B101" s="43"/>
+      <c r="C101" s="43"/>
+      <c r="D101" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="E101" s="43"/>
+    </row>
+    <row r="102" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="42"/>
+      <c r="B102" s="43"/>
+      <c r="C102" s="43"/>
+      <c r="D102" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="E102" s="43"/>
+    </row>
+    <row r="103" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="42"/>
+      <c r="B103" s="43"/>
+      <c r="C103" s="43"/>
+      <c r="D103" s="43" t="s">
+        <v>360</v>
+      </c>
+      <c r="E103" s="43"/>
+    </row>
+    <row r="104" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="42"/>
+      <c r="B104" s="43"/>
+      <c r="C104" s="43"/>
+      <c r="D104" s="43" t="s">
+        <v>493</v>
+      </c>
+      <c r="E104" s="43"/>
+    </row>
+    <row r="105" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="42"/>
+      <c r="B105" s="43"/>
+      <c r="C105" s="43"/>
+      <c r="D105" s="43" t="s">
+        <v>308</v>
+      </c>
+      <c r="E105" s="43"/>
+    </row>
+    <row r="106" spans="1:5" s="41" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="40"/>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="23">
         <v>12401</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B107" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C107" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D107" t="s">
         <v>229</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E107" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="23"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="23">
+    <row r="108" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="23"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="23">
         <v>12401</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B109" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C109" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D109" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E109" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D32" s="10" t="s">
+    <row r="110" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D110" s="10" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="23"/>
-      <c r="E33"/>
-    </row>
-    <row r="34" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="23"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="23"/>
-      <c r="D35" s="10"/>
-    </row>
-    <row r="36" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="23"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="23"/>
-      <c r="B37" s="10"/>
-      <c r="D37" s="10"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D38" s="10"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="23"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-    </row>
-    <row r="40" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
+    <row r="111" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="23"/>
+      <c r="E111"/>
+    </row>
+    <row r="112" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="23"/>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="23"/>
+      <c r="D113" s="10"/>
+    </row>
+    <row r="114" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="23"/>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="23"/>
+      <c r="B115" s="10"/>
+      <c r="D115" s="10"/>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D116" s="10"/>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="23"/>
+      <c r="B117" s="10"/>
+      <c r="C117" s="10"/>
+      <c r="D117" s="10"/>
+    </row>
+    <row r="118" spans="1:4" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="16"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
@@ -3984,6 +5573,2675 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04946517-378B-4098-A855-A25910B79684}">
+  <dimension ref="A1:J254"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="95.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>284</v>
+      </c>
+      <c r="D2" s="11"/>
+      <c r="E2" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="31">
+        <v>46048</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>285</v>
+      </c>
+      <c r="D3" s="11"/>
+      <c r="E3" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>286</v>
+      </c>
+      <c r="D4" s="11"/>
+      <c r="E4" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>288</v>
+      </c>
+      <c r="D5" s="11"/>
+      <c r="E5" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>289</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>290</v>
+      </c>
+      <c r="D7" s="11"/>
+      <c r="E7" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>292</v>
+      </c>
+      <c r="D8" s="11"/>
+      <c r="E8" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="C9" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>294</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="E10" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>295</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="E11" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="C12" s="36" t="s">
+        <v>296</v>
+      </c>
+      <c r="D12" s="11"/>
+      <c r="E12" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="C13" s="35" t="s">
+        <v>298</v>
+      </c>
+      <c r="D13" s="11"/>
+      <c r="E13" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="C14" s="35" t="s">
+        <v>299</v>
+      </c>
+      <c r="D14" s="11"/>
+      <c r="E14" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="C15" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="D15" s="11"/>
+      <c r="E15" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="C16" s="35" t="s">
+        <v>301</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="C17" s="35" t="s">
+        <v>302</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="C18" s="37" t="s">
+        <v>304</v>
+      </c>
+      <c r="D18" s="11"/>
+      <c r="E18" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="C19" s="35" t="s">
+        <v>305</v>
+      </c>
+      <c r="D19" s="11"/>
+      <c r="E19" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="C20" s="35" t="s">
+        <v>306</v>
+      </c>
+      <c r="D20" s="11"/>
+      <c r="E20" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="C21" s="37" t="s">
+        <v>307</v>
+      </c>
+      <c r="D21" s="11"/>
+      <c r="E21" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="C22" s="37" t="s">
+        <v>388</v>
+      </c>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="F22" s="31">
+        <v>45323</v>
+      </c>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>389</v>
+      </c>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="F23" s="31">
+        <v>45323</v>
+      </c>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="C24" s="35" t="s">
+        <v>309</v>
+      </c>
+      <c r="D24" s="11"/>
+      <c r="E24" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="C25" s="35" t="s">
+        <v>310</v>
+      </c>
+      <c r="D25" s="11"/>
+      <c r="E25" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="11" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="C26" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="D26" s="11"/>
+      <c r="E26" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="C27" s="38" t="s">
+        <v>313</v>
+      </c>
+      <c r="D27" s="11"/>
+      <c r="E27" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="C28" s="38" t="s">
+        <v>314</v>
+      </c>
+      <c r="D28" s="11"/>
+      <c r="E28" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>315</v>
+      </c>
+      <c r="D29" s="11"/>
+      <c r="E29" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+      <c r="J29" s="11" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="C30" s="38" t="s">
+        <v>316</v>
+      </c>
+      <c r="D30" s="11"/>
+      <c r="E30" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+      <c r="J30" s="11" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="C31" s="38" t="s">
+        <v>317</v>
+      </c>
+      <c r="D31" s="11"/>
+      <c r="E31" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
+      <c r="J31" s="11" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="C32" s="38" t="s">
+        <v>318</v>
+      </c>
+      <c r="D32" s="11"/>
+      <c r="E32" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+      <c r="J32" s="11" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="C33" s="38" t="s">
+        <v>319</v>
+      </c>
+      <c r="D33" s="11"/>
+      <c r="E33" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
+      <c r="J33" s="11" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="C34" s="38" t="s">
+        <v>320</v>
+      </c>
+      <c r="D34" s="11"/>
+      <c r="E34" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+      <c r="J34" s="11" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="C35" s="38" t="s">
+        <v>321</v>
+      </c>
+      <c r="D35" s="11"/>
+      <c r="E35" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11"/>
+      <c r="J35" s="11" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B36" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C36" s="44" t="s">
+        <v>322</v>
+      </c>
+      <c r="D36" s="27"/>
+      <c r="E36" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
+      <c r="I36" s="27"/>
+      <c r="J36" s="27" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B37" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C37" s="44" t="s">
+        <v>323</v>
+      </c>
+      <c r="D37" s="27"/>
+      <c r="E37" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="27"/>
+      <c r="J37" s="27" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C38" s="44" t="s">
+        <v>324</v>
+      </c>
+      <c r="D38" s="27"/>
+      <c r="E38" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="27"/>
+      <c r="J38" s="27" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B39" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C39" s="44" t="s">
+        <v>325</v>
+      </c>
+      <c r="D39" s="27"/>
+      <c r="E39" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F39" s="27"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="27"/>
+      <c r="J39" s="27" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B40" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C40" s="44" t="s">
+        <v>326</v>
+      </c>
+      <c r="D40" s="27"/>
+      <c r="E40" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="27" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B41" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C41" s="44" t="s">
+        <v>327</v>
+      </c>
+      <c r="D41" s="27"/>
+      <c r="E41" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="27"/>
+      <c r="J41" s="27" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B42" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C42" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="D42" s="27"/>
+      <c r="E42" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F42" s="27"/>
+      <c r="G42" s="27"/>
+      <c r="H42" s="27"/>
+      <c r="I42" s="27"/>
+      <c r="J42" s="27" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B43" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C43" s="44" t="s">
+        <v>329</v>
+      </c>
+      <c r="D43" s="27"/>
+      <c r="E43" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F43" s="27"/>
+      <c r="G43" s="27"/>
+      <c r="H43" s="27"/>
+      <c r="I43" s="27"/>
+      <c r="J43" s="27" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B44" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C44" s="44" t="s">
+        <v>330</v>
+      </c>
+      <c r="D44" s="27"/>
+      <c r="E44" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F44" s="27"/>
+      <c r="G44" s="27"/>
+      <c r="H44" s="27"/>
+      <c r="I44" s="27"/>
+      <c r="J44" s="27" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B45" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C45" s="44" t="s">
+        <v>331</v>
+      </c>
+      <c r="D45" s="27"/>
+      <c r="E45" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F45" s="27"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="27"/>
+      <c r="I45" s="27"/>
+      <c r="J45" s="27" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B46" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C46" s="44" t="s">
+        <v>332</v>
+      </c>
+      <c r="D46" s="27"/>
+      <c r="E46" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
+      <c r="I46" s="27"/>
+      <c r="J46" s="27" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B47" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="C47" s="45" t="s">
+        <v>333</v>
+      </c>
+      <c r="D47" s="27"/>
+      <c r="E47" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F47" s="27"/>
+      <c r="G47" s="27"/>
+      <c r="H47" s="27"/>
+      <c r="I47" s="27"/>
+      <c r="J47" s="27" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B48" s="27" t="s">
+        <v>393</v>
+      </c>
+      <c r="C48" s="45" t="s">
+        <v>392</v>
+      </c>
+      <c r="D48" s="27"/>
+      <c r="E48" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="F48" s="46">
+        <v>45349</v>
+      </c>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="27"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B49" s="27" t="s">
+        <v>394</v>
+      </c>
+      <c r="C49" s="47" t="s">
+        <v>362</v>
+      </c>
+      <c r="D49" s="27"/>
+      <c r="E49" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F49" s="27"/>
+      <c r="G49" s="27"/>
+      <c r="H49" s="27"/>
+      <c r="I49" s="27"/>
+      <c r="J49" s="27" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B50" s="27" t="s">
+        <v>395</v>
+      </c>
+      <c r="C50" s="47" t="s">
+        <v>372</v>
+      </c>
+      <c r="D50" s="27"/>
+      <c r="E50" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F50" s="27"/>
+      <c r="G50" s="27"/>
+      <c r="H50" s="27"/>
+      <c r="I50" s="27"/>
+      <c r="J50" s="27" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C51" s="38" t="s">
+        <v>374</v>
+      </c>
+      <c r="D51" s="11"/>
+      <c r="E51" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F51" s="11"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+      <c r="J51" s="11" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C52" s="38" t="s">
+        <v>375</v>
+      </c>
+      <c r="D52" s="11"/>
+      <c r="E52" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F52" s="11"/>
+      <c r="G52" s="11"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="11"/>
+      <c r="J52" s="11" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C53" s="38" t="s">
+        <v>376</v>
+      </c>
+      <c r="D53" s="11"/>
+      <c r="E53" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F53" s="11"/>
+      <c r="G53" s="11"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="11"/>
+      <c r="J53" s="11" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C54" s="38" t="s">
+        <v>377</v>
+      </c>
+      <c r="D54" s="11"/>
+      <c r="E54" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F54" s="11"/>
+      <c r="G54" s="11"/>
+      <c r="H54" s="11"/>
+      <c r="I54" s="11"/>
+      <c r="J54" s="11" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C55" s="38" t="s">
+        <v>378</v>
+      </c>
+      <c r="D55" s="11"/>
+      <c r="E55" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F55" s="11"/>
+      <c r="G55" s="11"/>
+      <c r="H55" s="11"/>
+      <c r="I55" s="11"/>
+      <c r="J55" s="11" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C56" s="38" t="s">
+        <v>379</v>
+      </c>
+      <c r="D56" s="11"/>
+      <c r="E56" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="11"/>
+      <c r="J56" s="11" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C57" s="38" t="s">
+        <v>380</v>
+      </c>
+      <c r="D57" s="11"/>
+      <c r="E57" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F57" s="11"/>
+      <c r="G57" s="11"/>
+      <c r="H57" s="11"/>
+      <c r="I57" s="11"/>
+      <c r="J57" s="11" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C58" s="38" t="s">
+        <v>381</v>
+      </c>
+      <c r="D58" s="11"/>
+      <c r="E58" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
+      <c r="J58" s="11" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C59" s="38" t="s">
+        <v>382</v>
+      </c>
+      <c r="D59" s="11"/>
+      <c r="E59" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F59" s="11"/>
+      <c r="G59" s="11"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
+      <c r="J59" s="11" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C60" s="38" t="s">
+        <v>383</v>
+      </c>
+      <c r="D60" s="11"/>
+      <c r="E60" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F60" s="11"/>
+      <c r="G60" s="11"/>
+      <c r="H60" s="11"/>
+      <c r="I60" s="11"/>
+      <c r="J60" s="11" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C61" s="38" t="s">
+        <v>384</v>
+      </c>
+      <c r="D61" s="11"/>
+      <c r="E61" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F61" s="11"/>
+      <c r="G61" s="11"/>
+      <c r="H61" s="11"/>
+      <c r="I61" s="11"/>
+      <c r="J61" s="11" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="C62" s="38" t="s">
+        <v>385</v>
+      </c>
+      <c r="D62" s="11"/>
+      <c r="E62" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F62" s="11"/>
+      <c r="G62" s="11"/>
+      <c r="H62" s="11"/>
+      <c r="I62" s="11"/>
+      <c r="J62" s="11" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B63" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C63" s="39" t="s">
+        <v>335</v>
+      </c>
+      <c r="D63" s="11"/>
+      <c r="E63" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F63" s="11"/>
+      <c r="G63" s="11"/>
+      <c r="H63" s="11"/>
+      <c r="I63" s="11"/>
+      <c r="J63" s="11" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C64" s="39" t="s">
+        <v>336</v>
+      </c>
+      <c r="D64" s="11"/>
+      <c r="E64" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F64" s="11"/>
+      <c r="G64" s="11"/>
+      <c r="H64" s="11"/>
+      <c r="I64" s="11"/>
+      <c r="J64" s="11" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C65" s="39" t="s">
+        <v>337</v>
+      </c>
+      <c r="D65" s="11"/>
+      <c r="E65" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F65" s="11"/>
+      <c r="G65" s="11"/>
+      <c r="H65" s="11"/>
+      <c r="I65" s="11"/>
+      <c r="J65" s="11" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C66" s="39" t="s">
+        <v>338</v>
+      </c>
+      <c r="D66" s="11"/>
+      <c r="E66" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F66" s="11"/>
+      <c r="G66" s="11"/>
+      <c r="H66" s="11"/>
+      <c r="I66" s="11"/>
+      <c r="J66" s="11" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C67" s="39" t="s">
+        <v>339</v>
+      </c>
+      <c r="D67" s="11"/>
+      <c r="E67" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F67" s="11"/>
+      <c r="G67" s="11"/>
+      <c r="H67" s="11"/>
+      <c r="I67" s="11"/>
+      <c r="J67" s="11" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B68" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C68" s="39" t="s">
+        <v>340</v>
+      </c>
+      <c r="D68" s="11"/>
+      <c r="E68" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F68" s="11"/>
+      <c r="G68" s="11"/>
+      <c r="H68" s="11"/>
+      <c r="I68" s="11"/>
+      <c r="J68" s="11" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C69" s="39" t="s">
+        <v>341</v>
+      </c>
+      <c r="D69" s="11"/>
+      <c r="E69" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F69" s="11"/>
+      <c r="G69" s="11"/>
+      <c r="H69" s="11"/>
+      <c r="I69" s="11"/>
+      <c r="J69" s="11" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C70" s="39" t="s">
+        <v>342</v>
+      </c>
+      <c r="D70" s="11"/>
+      <c r="E70" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F70" s="11"/>
+      <c r="G70" s="11"/>
+      <c r="H70" s="11"/>
+      <c r="I70" s="11"/>
+      <c r="J70" s="11" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C71" s="39" t="s">
+        <v>343</v>
+      </c>
+      <c r="D71" s="11"/>
+      <c r="E71" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F71" s="11"/>
+      <c r="G71" s="11"/>
+      <c r="H71" s="11"/>
+      <c r="I71" s="11"/>
+      <c r="J71" s="11" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A72" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C72" s="39" t="s">
+        <v>344</v>
+      </c>
+      <c r="D72" s="11"/>
+      <c r="E72" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F72" s="11"/>
+      <c r="G72" s="11"/>
+      <c r="H72" s="11"/>
+      <c r="I72" s="11"/>
+      <c r="J72" s="11" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B73" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C73" s="39" t="s">
+        <v>345</v>
+      </c>
+      <c r="D73" s="11"/>
+      <c r="E73" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F73" s="11"/>
+      <c r="G73" s="11"/>
+      <c r="H73" s="11"/>
+      <c r="I73" s="11"/>
+      <c r="J73" s="11" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C74" s="39" t="s">
+        <v>346</v>
+      </c>
+      <c r="D74" s="11"/>
+      <c r="E74" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F74" s="11"/>
+      <c r="G74" s="11"/>
+      <c r="H74" s="11"/>
+      <c r="I74" s="11"/>
+      <c r="J74" s="11" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B75" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C75" s="34" t="s">
+        <v>348</v>
+      </c>
+      <c r="D75" s="11"/>
+      <c r="E75" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F75" s="11"/>
+      <c r="G75" s="11"/>
+      <c r="H75" s="11"/>
+      <c r="I75" s="11"/>
+      <c r="J75" s="11" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C76" s="34" t="s">
+        <v>349</v>
+      </c>
+      <c r="D76" s="11"/>
+      <c r="E76" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F76" s="11"/>
+      <c r="G76" s="11"/>
+      <c r="H76" s="11"/>
+      <c r="I76" s="11"/>
+      <c r="J76" s="11" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C77" s="34" t="s">
+        <v>350</v>
+      </c>
+      <c r="D77" s="11"/>
+      <c r="E77" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F77" s="11"/>
+      <c r="G77" s="11"/>
+      <c r="H77" s="11"/>
+      <c r="I77" s="11"/>
+      <c r="J77" s="11" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B78" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C78" s="34" t="s">
+        <v>351</v>
+      </c>
+      <c r="D78" s="11"/>
+      <c r="E78" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F78" s="11"/>
+      <c r="G78" s="11"/>
+      <c r="H78" s="11"/>
+      <c r="I78" s="11"/>
+      <c r="J78" s="11" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B79" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C79" s="34" t="s">
+        <v>352</v>
+      </c>
+      <c r="D79" s="11"/>
+      <c r="E79" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F79" s="11"/>
+      <c r="G79" s="11"/>
+      <c r="H79" s="11"/>
+      <c r="I79" s="11"/>
+      <c r="J79" s="11" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C80" s="34" t="s">
+        <v>353</v>
+      </c>
+      <c r="D80" s="11"/>
+      <c r="E80" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F80" s="11"/>
+      <c r="G80" s="11"/>
+      <c r="H80" s="11"/>
+      <c r="I80" s="11"/>
+      <c r="J80" s="11" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B81" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C81" s="34" t="s">
+        <v>354</v>
+      </c>
+      <c r="D81" s="11"/>
+      <c r="E81" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F81" s="11"/>
+      <c r="G81" s="11"/>
+      <c r="H81" s="11"/>
+      <c r="I81" s="11"/>
+      <c r="J81" s="11" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C82" s="34" t="s">
+        <v>355</v>
+      </c>
+      <c r="D82" s="11"/>
+      <c r="E82" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F82" s="11"/>
+      <c r="G82" s="11"/>
+      <c r="H82" s="11"/>
+      <c r="I82" s="11"/>
+      <c r="J82" s="11" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A83" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B83" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C83" s="34" t="s">
+        <v>356</v>
+      </c>
+      <c r="D83" s="11"/>
+      <c r="E83" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F83" s="11"/>
+      <c r="G83" s="11"/>
+      <c r="H83" s="11"/>
+      <c r="I83" s="11"/>
+      <c r="J83" s="11" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B84" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C84" s="34" t="s">
+        <v>357</v>
+      </c>
+      <c r="D84" s="11"/>
+      <c r="E84" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F84" s="11"/>
+      <c r="G84" s="11"/>
+      <c r="H84" s="11"/>
+      <c r="I84" s="11"/>
+      <c r="J84" s="11" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B85" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C85" s="34" t="s">
+        <v>358</v>
+      </c>
+      <c r="D85" s="11"/>
+      <c r="E85" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F85" s="11"/>
+      <c r="G85" s="11"/>
+      <c r="H85" s="11"/>
+      <c r="I85" s="11"/>
+      <c r="J85" s="11" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B86" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C86" s="39" t="s">
+        <v>359</v>
+      </c>
+      <c r="D86" s="11"/>
+      <c r="E86" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F86" s="11"/>
+      <c r="G86" s="11"/>
+      <c r="H86" s="11"/>
+      <c r="I86" s="11"/>
+      <c r="J86" s="11" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B87" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="C87" s="37" t="s">
+        <v>361</v>
+      </c>
+      <c r="D87" s="11"/>
+      <c r="E87" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F87" s="11"/>
+      <c r="G87" s="11"/>
+      <c r="H87" s="11"/>
+      <c r="I87" s="11"/>
+      <c r="J87" s="11" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B88" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="C88" s="37" t="s">
+        <v>391</v>
+      </c>
+      <c r="D88" s="11"/>
+      <c r="E88" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="F88" s="31">
+        <v>45474</v>
+      </c>
+      <c r="G88" s="11"/>
+      <c r="H88" s="11"/>
+      <c r="I88" s="11"/>
+      <c r="J88" s="11"/>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B89" s="11" t="s">
+        <v>370</v>
+      </c>
+      <c r="C89" s="38" t="s">
+        <v>371</v>
+      </c>
+      <c r="D89" s="11"/>
+      <c r="E89" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F89" s="11"/>
+      <c r="G89" s="11"/>
+      <c r="H89" s="11"/>
+      <c r="I89" s="11"/>
+      <c r="J89" s="11" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B90" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="C90" s="37" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="11"/>
+      <c r="E90" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F90" s="11"/>
+      <c r="G90" s="11"/>
+      <c r="H90" s="11"/>
+      <c r="I90" s="11"/>
+      <c r="J90" s="11" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A91" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B91" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="C91" s="34" t="s">
+        <v>363</v>
+      </c>
+      <c r="D91" s="11"/>
+      <c r="E91" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F91" s="11"/>
+      <c r="G91" s="11"/>
+      <c r="H91" s="11"/>
+      <c r="I91" s="11"/>
+      <c r="J91" s="11" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A92" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B92" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="C92" s="34" t="s">
+        <v>364</v>
+      </c>
+      <c r="D92" s="11"/>
+      <c r="E92" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F92" s="11"/>
+      <c r="G92" s="11"/>
+      <c r="H92" s="11"/>
+      <c r="I92" s="11"/>
+      <c r="J92" s="11" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A93" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B93" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="C93" s="34" t="s">
+        <v>365</v>
+      </c>
+      <c r="D93" s="11"/>
+      <c r="E93" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F93" s="11"/>
+      <c r="G93" s="11"/>
+      <c r="H93" s="11"/>
+      <c r="I93" s="11"/>
+      <c r="J93" s="11" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A94" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B94" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="C94" s="34" t="s">
+        <v>366</v>
+      </c>
+      <c r="D94" s="11"/>
+      <c r="E94" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F94" s="11"/>
+      <c r="G94" s="11"/>
+      <c r="H94" s="11"/>
+      <c r="I94" s="11"/>
+      <c r="J94" s="11" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A95" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B95" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="C95" s="34" t="s">
+        <v>367</v>
+      </c>
+      <c r="D95" s="11"/>
+      <c r="E95" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F95" s="11"/>
+      <c r="G95" s="11"/>
+      <c r="H95" s="11"/>
+      <c r="I95" s="11"/>
+      <c r="J95" s="11" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A96" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B96" s="11" t="s">
+        <v>368</v>
+      </c>
+      <c r="C96" s="39" t="s">
+        <v>369</v>
+      </c>
+      <c r="D96" s="11"/>
+      <c r="E96" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F96" s="11"/>
+      <c r="G96" s="11"/>
+      <c r="H96" s="11" t="s">
+        <v>387</v>
+      </c>
+      <c r="I96" s="11"/>
+      <c r="J96" s="11" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B97" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C97" s="39" t="s">
+        <v>335</v>
+      </c>
+      <c r="D97" s="11"/>
+      <c r="E97" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F97" s="11"/>
+      <c r="G97" s="11"/>
+      <c r="H97" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I97" s="11"/>
+      <c r="J97" s="11" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B98" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C98" s="39" t="s">
+        <v>336</v>
+      </c>
+      <c r="D98" s="11"/>
+      <c r="E98" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F98" s="11"/>
+      <c r="G98" s="11"/>
+      <c r="H98" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I98" s="11"/>
+      <c r="J98" s="11" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B99" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C99" s="39" t="s">
+        <v>337</v>
+      </c>
+      <c r="D99" s="11"/>
+      <c r="E99" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F99" s="11"/>
+      <c r="G99" s="11"/>
+      <c r="H99" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I99" s="11"/>
+      <c r="J99" s="11" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B100" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C100" s="39" t="s">
+        <v>338</v>
+      </c>
+      <c r="D100" s="11"/>
+      <c r="E100" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F100" s="11"/>
+      <c r="G100" s="11"/>
+      <c r="H100" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I100" s="11"/>
+      <c r="J100" s="11" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B101" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C101" s="39" t="s">
+        <v>339</v>
+      </c>
+      <c r="D101" s="11"/>
+      <c r="E101" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F101" s="11"/>
+      <c r="G101" s="11"/>
+      <c r="H101" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I101" s="11"/>
+      <c r="J101" s="11" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B102" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C102" s="39" t="s">
+        <v>340</v>
+      </c>
+      <c r="D102" s="11"/>
+      <c r="E102" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F102" s="11"/>
+      <c r="G102" s="11"/>
+      <c r="H102" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I102" s="11"/>
+      <c r="J102" s="11" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B103" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C103" s="39" t="s">
+        <v>341</v>
+      </c>
+      <c r="D103" s="11"/>
+      <c r="E103" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F103" s="11"/>
+      <c r="G103" s="11"/>
+      <c r="H103" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I103" s="11"/>
+      <c r="J103" s="11" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B104" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C104" s="39" t="s">
+        <v>342</v>
+      </c>
+      <c r="D104" s="11"/>
+      <c r="E104" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F104" s="11"/>
+      <c r="G104" s="11"/>
+      <c r="H104" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I104" s="11"/>
+      <c r="J104" s="11" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B105" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C105" s="39" t="s">
+        <v>343</v>
+      </c>
+      <c r="D105" s="11"/>
+      <c r="E105" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F105" s="11"/>
+      <c r="G105" s="11"/>
+      <c r="H105" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I105" s="11"/>
+      <c r="J105" s="11" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B106" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C106" s="39" t="s">
+        <v>344</v>
+      </c>
+      <c r="D106" s="11"/>
+      <c r="E106" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F106" s="11"/>
+      <c r="G106" s="11"/>
+      <c r="H106" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I106" s="11"/>
+      <c r="J106" s="11" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B107" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C107" s="39" t="s">
+        <v>345</v>
+      </c>
+      <c r="D107" s="11"/>
+      <c r="E107" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F107" s="11"/>
+      <c r="G107" s="11"/>
+      <c r="H107" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I107" s="11"/>
+      <c r="J107" s="11" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B108" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="C108" s="39" t="s">
+        <v>346</v>
+      </c>
+      <c r="D108" s="11"/>
+      <c r="E108" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F108" s="11"/>
+      <c r="G108" s="11"/>
+      <c r="H108" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I108" s="11"/>
+      <c r="J108" s="11" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B109" s="11" t="s">
+        <v>400</v>
+      </c>
+      <c r="C109" s="37" t="s">
+        <v>361</v>
+      </c>
+      <c r="D109" s="11"/>
+      <c r="E109" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F109" s="11"/>
+      <c r="G109" s="11"/>
+      <c r="H109" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="I109" s="11"/>
+      <c r="J109" s="11" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B110" s="11" t="s">
+        <v>493</v>
+      </c>
+      <c r="C110" s="11" t="s">
+        <v>494</v>
+      </c>
+      <c r="D110" s="11"/>
+      <c r="E110" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F110" s="31"/>
+      <c r="G110" s="11"/>
+      <c r="H110" s="11" t="s">
+        <v>497</v>
+      </c>
+      <c r="I110" s="11"/>
+      <c r="J110" s="11" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B111" s="11" t="s">
+        <v>493</v>
+      </c>
+      <c r="C111" s="11" t="s">
+        <v>495</v>
+      </c>
+      <c r="E111" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="H111" s="11" t="s">
+        <v>497</v>
+      </c>
+      <c r="J111" s="10" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="18">
+        <v>10202</v>
+      </c>
+      <c r="B112" s="11" t="s">
+        <v>493</v>
+      </c>
+      <c r="C112" s="11" t="s">
+        <v>496</v>
+      </c>
+      <c r="E112" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="H112" s="11" t="s">
+        <v>497</v>
+      </c>
+      <c r="J112" s="10" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="113" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="114" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="115" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="116" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="117" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="118" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="119" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="120" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="121" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="122" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="123" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="124" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="125" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="126" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="127" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="128" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="129" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="130" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="131" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="132" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="133" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="134" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="135" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="136" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="137" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="138" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="139" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="140" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="141" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="142" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="143" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="144" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="145" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="146" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="147" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="148" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="149" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="150" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="151" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="152" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="153" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="154" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="155" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="156" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="157" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="158" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="159" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="160" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="161" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="162" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="163" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="164" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="165" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="166" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="167" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="168" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="169" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="170" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="171" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="172" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="173" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="174" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="175" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="176" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="177" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="178" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="179" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="180" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="181" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="182" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="183" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="184" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="185" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="186" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="187" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="188" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="189" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="190" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="191" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="192" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="193" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="194" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="195" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="196" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="197" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="198" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="199" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="200" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="201" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="202" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="203" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="204" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="205" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="206" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="207" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="208" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="209" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="210" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="212" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="213" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="216" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="217" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F217"/>
+    </row>
+    <row r="218" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="223" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="224" spans="6:6" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="225" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="226" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="227" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="228" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="229" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="230" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="231" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="232" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="233" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="234" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="235" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="236" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="237" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="238" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="239" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="240" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="241" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="242" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="243" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="244" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="245" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="246" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="247" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="248" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="249" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="250" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="251" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="252" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="253" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="254" s="10" customFormat="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E45063F7-9C44-48AD-A336-67B5B01C844C}">
   <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>